<commit_message>
feat(beneficiaries): implementa barra de progresso na exportacao e melhora interceptors
- Exportação: Adicionado modal com barra de progresso visual simulada não-linear para a exportação de planilhas e correção na cor CSS da barra.

- Acessibilidade: Integrado o LiveAnnouncer para anunciar o progresso gradativo (ex: 20%, 50%, concluído) aos leitores de tela.

- Interceptors (Auth): O token JWT agora é injetado apenas nas rotas da API interna do projeto, evitando bloqueios CORS com APIs públicas.

- Interceptors (Error): Erros globais via Toast agora são disparados somente para a API interna, prevenindo mensagens genéricas (ex: Servidor Fora do Ar) em buscas como ViaCEP.

- ViaCEP: Adicionado validação no formulário que captura 'erro: true' da API externa, invalidando visualmente o campo de CEP na UI.
</commit_message>
<xml_diff>
--- a/src/assets/modelo-importacao-alunos.xlsx
+++ b/src/assets/modelo-importacao-alunos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PI-5\Braille-Frontend\src\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DACF511-22B7-440C-B304-116CEDFD17D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33D41E79-CACD-4A01-97E4-3AB02988D79B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -240,7 +240,7 @@
     <t xml:space="preserve">Ex: 11.111.111 </t>
   </si>
   <si>
-    <t xml:space="preserve">CPF </t>
+    <t>CPF</t>
   </si>
 </sst>
 </file>
@@ -873,55 +873,60 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:Y2" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <ignoredErrors>
-    <ignoredError sqref="Q2:Y2 D2:O2 A2" numberStoredAsText="1"/>
+    <ignoredError sqref="T2:W2 N2:O2 L2" numberStoredAsText="1"/>
   </ignoredErrors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="7">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="8">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{19035003-A070-4FF7-BD0C-8418E5EC12A0}">
           <x14:formula1>
             <xm:f>Instruções!$E$3:$E$5</xm:f>
           </x14:formula1>
-          <xm:sqref>I3:I6457</xm:sqref>
+          <xm:sqref>Q3:Q1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B3928D14-F069-43F0-B787-22BED2FA21D5}">
           <x14:formula1>
             <xm:f>Instruções!$A$10:$A$11</xm:f>
           </x14:formula1>
-          <xm:sqref>J3:J6457</xm:sqref>
+          <xm:sqref>R3:R1048576</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{C0860636-1AC8-4C3F-914C-34578DF95BBA}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{E5A8A6B5-9503-40D9-8734-778FC837BB6A}">
           <x14:formula1>
-            <xm:f>Instruções!$E$10:$E$17</xm:f>
+            <xm:f>Instruções!$I$3:$I$6</xm:f>
           </x14:formula1>
-          <xm:sqref>K3:K6457</xm:sqref>
+          <xm:sqref>Y3:Y1048576</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F13234A7-3F0D-4F57-A847-CE63B53E5D99}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{C90C44D7-77A9-49A0-8B19-39D588AC2DD8}">
           <x14:formula1>
-            <xm:f>Instruções!$G$3:$G$5</xm:f>
+            <xm:f>Instruções!$A$3:$A$6</xm:f>
           </x14:formula1>
-          <xm:sqref>M3:M6457</xm:sqref>
+          <xm:sqref>E3:E1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{E2412CD7-F840-4B18-9EE0-0EB2C86EBA0E}">
+          <x14:formula1>
+            <xm:f>Instruções!$C$3:$C$7</xm:f>
+          </x14:formula1>
+          <xm:sqref>F3:F1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{11DDE071-7C92-4D37-9379-4ADFD1483A76}">
           <x14:formula1>
             <xm:f>Instruções!$C$10:$C$11</xm:f>
           </x14:formula1>
-          <xm:sqref>P3:P6457</xm:sqref>
+          <xm:sqref>X3:X1048576</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{E5A8A6B5-9503-40D9-8734-778FC837BB6A}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{6D0657BB-C840-4BB2-A2C7-C72D4E8C1860}">
           <x14:formula1>
-            <xm:f>Instruções!$I$3:$I$6</xm:f>
+            <xm:f>Instruções!$E$10:$E$17</xm:f>
           </x14:formula1>
-          <xm:sqref>Q3:Q6457</xm:sqref>
+          <xm:sqref>S3:S1048576</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{BD25C12D-0A9B-467C-A431-536F15A75328}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{5F941123-C233-4C9E-9BF1-8D0385A99488}">
           <x14:formula1>
             <xm:f>Instruções!$G$10:$G$15</xm:f>
           </x14:formula1>
-          <xm:sqref>H3:H3595</xm:sqref>
+          <xm:sqref>P3:P1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>